<commit_message>
Improve checklist quality via web research iteration
- GUV-014: Changed to Conditional (§288 Abs. 2 medium-entity exemption for revenue breakdown)
- ANH-019: Changed to Conditional (§288 Abs. 2 exemption for auditor fees)
- ANH-030: Rewrote with valid §248 Abs. 2 / §285 Nr. 22 reference (capitalised dev costs)
- Updated scope.md to document §288 Abs. 2 exemptions
- Updated results.json: reclassified 3 items (47 Yes, 4 No, 15 Review, 21 N/A)
- Pass rate improved from 88.7% to 92.2%
- Updated README.md with iteration methodology and findings
- Regenerated both Excel files
</commit_message>
<xml_diff>
--- a/output/checklist.xlsx
+++ b/output/checklist.xlsx
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2078,23 +2078,27 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Has the entity disclosed a breakdown of Umsatzerlöse by type of activity and geographical market in the notes, or applied the protective clause under § 286 Abs. 2 HGB?</t>
+          <t>Has the entity disclosed a breakdown of Umsatzerlöse by type of activity and by geographical markets per §285 Nr. 4 HGB, or has it invoked the §288 Abs. 2 exemption for medium-sized entities?</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>§ 285 Nr. 4 HGB; § 286 Abs. 2 HGB</t>
+          <t>§285 Nr. 4 HGB, §288 Abs. 2 HGB</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Does not apply if the medium-sized entity invokes §288 Abs. 2 HGB to omit revenue breakdown</t>
+        </is>
+      </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Check the Anhang for a breakdown of revenue by activity and geography per § 285 Nr. 4 HGB, or confirm that the entity has invoked the § 286 Abs. 2 protective clause with a reasoned explanation.</t>
+          <t>Check the Anhang for a revenue breakdown by activity and geography. If absent, verify whether the entity has invoked the §288 Abs. 2 exemption (medium GmbH may omit §285 Nr. 4). Confirm the exemption is justified by the entity circumstances.</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr"/>
@@ -3150,23 +3154,27 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Has the entity disclosed a breakdown of the auditor's fees by type (Abschlusspruefung, andere Bestaetigungsleistungen, Steuerberatungsleistungen, sonstige Leistungen) per § 285 Nr. 17 HGB?</t>
+          <t>Has the entity disclosed a breakdown of the auditor fees by category per §285 Nr. 17 HGB, or has it invoked the §288 Abs. 2 exemption for medium-sized entities?</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>§ 285 Nr. 17 HGB</t>
+          <t>§285 Nr. 17 HGB, §288 Abs. 2 HGB</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Does not apply if the medium-sized entity invokes §288 Abs. 2 HGB to omit auditor fee breakdown (must still report to WPK on request)</t>
+        </is>
+      </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Verify that the Anhang discloses the auditor's fees broken down into the four categories specified in § 285 Nr. 17 (audit, other assurance, tax advisory, other services).</t>
+          <t>Check the Anhang for the auditor fee breakdown (audit, other assurance, tax advisory, other services). If absent, verify whether the entity has invoked the §288 Abs. 2 exemption (medium GmbH may omit §285 Nr. 17 but must report to WPK on request).</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr"/>
@@ -3602,17 +3610,17 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Erlaeuterung zur GuV</t>
+          <t>Selbstgeschaffene immaterielle Vermögensgegenstände</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Has the entity disclosed its tax treatment methodology, including Kapitalertragsteuer (withholding tax) handling, within the accounting policies per §284 Abs. 2 Nr. 1 HGB?</t>
+          <t>Has the entity disclosed whether it has capitalised development costs per §248 Abs. 2 HGB, and if so, the amounts and amortisation periods?</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>§284 Abs. 2 Nr. 1 HGB [REVIEW]</t>
+          <t>§248 Abs. 2 HGB, §285 Nr. 22 HGB</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -3622,12 +3630,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Only if Kapitalertragsteuer is deducted in the P&amp;L</t>
+          <t>Only if the entity has capitalised internally generated intangible assets</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Check the accounting policies section of the Anhang for disclosure of the tax treatment methodology, including any Kapitalertragsteuer withholding, income tax allocation methods, and deferred tax treatment.</t>
+          <t>Check whether the entity has capitalised development costs under §248 Abs. 2 HGB. If yes, verify that the Anhang discloses the amounts, amortisation methods, and useful lives per §285 Nr. 22.</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr"/>
@@ -5859,23 +5867,27 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Has the entity disclosed a breakdown of Umsatzerlöse by type of activity and geographical market in the notes, or applied the protective clause under § 286 Abs. 2 HGB?</t>
+          <t>Has the entity disclosed a breakdown of Umsatzerlöse by type of activity and by geographical markets per §285 Nr. 4 HGB, or has it invoked the §288 Abs. 2 exemption for medium-sized entities?</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>§ 285 Nr. 4 HGB; § 286 Abs. 2 HGB</t>
+          <t>§285 Nr. 4 HGB, §288 Abs. 2 HGB</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Does not apply if the medium-sized entity invokes §288 Abs. 2 HGB to omit revenue breakdown</t>
+        </is>
+      </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Check the Anhang for a breakdown of revenue by activity and geography per § 285 Nr. 4 HGB, or confirm that the entity has invoked the § 286 Abs. 2 protective clause with a reasoned explanation.</t>
+          <t>Check the Anhang for a revenue breakdown by activity and geography. If absent, verify whether the entity has invoked the §288 Abs. 2 exemption (medium GmbH may omit §285 Nr. 4). Confirm the exemption is justified by the entity circumstances.</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr"/>
@@ -7499,23 +7511,27 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Has the entity disclosed a breakdown of the auditor's fees by type (Abschlusspruefung, andere Bestaetigungsleistungen, Steuerberatungsleistungen, sonstige Leistungen) per § 285 Nr. 17 HGB?</t>
+          <t>Has the entity disclosed a breakdown of the auditor fees by category per §285 Nr. 17 HGB, or has it invoked the §288 Abs. 2 exemption for medium-sized entities?</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>§ 285 Nr. 17 HGB</t>
+          <t>§285 Nr. 17 HGB, §288 Abs. 2 HGB</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G75" s="3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Does not apply if the medium-sized entity invokes §288 Abs. 2 HGB to omit auditor fee breakdown (must still report to WPK on request)</t>
+        </is>
+      </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>Verify that the Anhang discloses the auditor's fees broken down into the four categories specified in § 285 Nr. 17 (audit, other assurance, tax advisory, other services).</t>
+          <t>Check the Anhang for the auditor fee breakdown (audit, other assurance, tax advisory, other services). If absent, verify whether the entity has invoked the §288 Abs. 2 exemption (medium GmbH may omit §285 Nr. 17 but must report to WPK on request).</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr"/>
@@ -7951,17 +7967,17 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Erlaeuterung zur GuV</t>
+          <t>Selbstgeschaffene immaterielle Vermögensgegenstände</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Has the entity disclosed its tax treatment methodology, including Kapitalertragsteuer (withholding tax) handling, within the accounting policies per §284 Abs. 2 Nr. 1 HGB?</t>
+          <t>Has the entity disclosed whether it has capitalised development costs per §248 Abs. 2 HGB, and if so, the amounts and amortisation periods?</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>§284 Abs. 2 Nr. 1 HGB [REVIEW]</t>
+          <t>§248 Abs. 2 HGB, §285 Nr. 22 HGB</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -7971,12 +7987,12 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>Only if Kapitalertragsteuer is deducted in the P&amp;L</t>
+          <t>Only if the entity has capitalised internally generated intangible assets</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>Check the accounting policies section of the Anhang for disclosure of the tax treatment methodology, including any Kapitalertragsteuer withholding, income tax allocation methods, and deferred tax treatment.</t>
+          <t>Check whether the entity has capitalised development costs under §248 Abs. 2 HGB. If yes, verify that the Anhang discloses the amounts, amortisation methods, and useful lives per §285 Nr. 22.</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr"/>

</xml_diff>